<commit_message>
Project excel generator done
</commit_message>
<xml_diff>
--- a/Solution1/ProjectClock.MVC/wwwroot/excel_templates/template_user.xlsx
+++ b/Solution1/ProjectClock.MVC/wwwroot/excel_templates/template_user.xlsx
@@ -62,7 +62,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm-dd-yyyy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -76,7 +76,6 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
-    <font/>
     <font>
       <b/>
       <i/>
@@ -120,121 +119,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF3C78D8"/>
+        <bgColor rgb="FF3C78D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF6D9EEB"/>
         <bgColor rgb="FF6D9EEB"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA4C2F4"/>
-        <bgColor rgb="FFA4C2F4"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border/>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
-    <border>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
-    <border>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-    </border>
-    <border>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="6" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="7" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="7" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="8" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -457,63 +384,59 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="7" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="6">
         <v>35805.0</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5">
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
     </row>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>

</xml_diff>